<commit_message>
excel reto 1, reto 2 faltante
</commit_message>
<xml_diff>
--- a/Docs/ISIS1225-TablasDatosReto2.xlsx
+++ b/Docs/ISIS1225-TablasDatosReto2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f37e920cb68ed4a8/Desktop/Reto2-G03/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{4A5DBDDE-59DE-4983-A5DD-216DD4370536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CE162CA-726A-4580-81E1-998AC705562F}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{4A5DBDDE-59DE-4983-A5DD-216DD4370536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3F9D279-734E-4354-9D33-39B9177A17B5}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
@@ -227,13 +227,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -893,31 +893,31 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.1147</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>9.3816000000000006</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>17.235299999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>28.8857</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>48.176900000000003</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>51.407699999999998</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>68.365899999999996</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>85.055099999999996</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>90.106300000000005</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>127.274</c:v>
@@ -2003,7 +2003,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8674100" cy="6286500"/>
+    <xdr:ext cx="9296400" cy="6070600"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -2401,14 +2401,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="14.25" customHeight="1">
-      <c r="C1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="C1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:9" s="5" customFormat="1" ht="28">
       <c r="A2" s="4" t="s">
@@ -2445,23 +2445,23 @@
         <v>10000</v>
       </c>
       <c r="C3" s="3">
-        <v>0</v>
+        <v>0.1147</v>
       </c>
       <c r="D3" s="3">
-        <v>0</v>
+        <v>7.2500200000000001E-2</v>
       </c>
       <c r="E3" s="3">
-        <v>0</v>
+        <v>0.1249</v>
       </c>
       <c r="F3" s="3">
-        <v>0</v>
+        <v>0.1101</v>
       </c>
       <c r="G3" s="3">
-        <v>0</v>
+        <v>0.13919999999999999</v>
       </c>
       <c r="H3" s="4">
         <f>AVERAGE(Table1[[#This Row],[Tiempo1]:[Tiempo5]])</f>
-        <v>0</v>
+        <v>0.11228004</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="5" customFormat="1" ht="14">
@@ -2501,23 +2501,23 @@
         <v>30000</v>
       </c>
       <c r="C5" s="3">
-        <v>0</v>
+        <v>17.235299999999999</v>
       </c>
       <c r="D5" s="3">
-        <v>0</v>
+        <v>16.161000000000001</v>
       </c>
       <c r="E5" s="3">
-        <v>0</v>
+        <v>17.22</v>
       </c>
       <c r="F5" s="3">
-        <v>0</v>
+        <v>18.523</v>
       </c>
       <c r="G5" s="3">
-        <v>0</v>
+        <v>17.043299999999999</v>
       </c>
       <c r="H5" s="4">
         <f>AVERAGE(Table1[[#This Row],[Tiempo1]:[Tiempo5]])</f>
-        <v>0</v>
+        <v>17.236519999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2557,23 +2557,23 @@
         <v>50000</v>
       </c>
       <c r="C7" s="3">
-        <v>0</v>
+        <v>48.176900000000003</v>
       </c>
       <c r="D7" s="3">
-        <v>0</v>
+        <v>47.979799999999997</v>
       </c>
       <c r="E7" s="3">
-        <v>0</v>
+        <v>50.816699999999997</v>
       </c>
       <c r="F7" s="3">
-        <v>0</v>
+        <v>47.734999999999999</v>
       </c>
       <c r="G7" s="3">
-        <v>0</v>
+        <v>46.3172</v>
       </c>
       <c r="H7" s="4">
         <f>AVERAGE(Table1[[#This Row],[Tiempo1]:[Tiempo5]])</f>
-        <v>0</v>
+        <v>48.205120000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2613,23 +2613,23 @@
         <v>70000</v>
       </c>
       <c r="C9" s="3">
-        <v>0</v>
+        <v>68.365899999999996</v>
       </c>
       <c r="D9" s="3">
-        <v>0</v>
+        <v>66.650899999999993</v>
       </c>
       <c r="E9" s="3">
-        <v>0</v>
+        <v>67.638099999999994</v>
       </c>
       <c r="F9" s="3">
-        <v>0</v>
+        <v>64.061700099999996</v>
       </c>
       <c r="G9" s="3">
-        <v>0</v>
+        <v>66.135999999999996</v>
       </c>
       <c r="H9" s="4">
         <f>AVERAGE(Table1[[#This Row],[Tiempo1]:[Tiempo5]])</f>
-        <v>0</v>
+        <v>66.570520020000004</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2659,7 +2659,7 @@
         <f>AVERAGE(Table1[[#This Row],[Tiempo1]:[Tiempo5]])</f>
         <v>82.988560000000007</v>
       </c>
-      <c r="I10" s="11"/>
+      <c r="I10" s="9"/>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="2">
@@ -2670,23 +2670,23 @@
         <v>90000</v>
       </c>
       <c r="C11" s="3">
-        <v>0</v>
+        <v>90.106300000000005</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>89.195300000000003</v>
       </c>
       <c r="E11" s="3">
-        <v>0</v>
+        <v>87.213399999999993</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>88.127799999999993</v>
       </c>
       <c r="G11" s="3">
-        <v>0</v>
+        <v>100.12730000000001</v>
       </c>
       <c r="H11" s="4">
         <f>AVERAGE(Table1[[#This Row],[Tiempo1]:[Tiempo5]])</f>
-        <v>0</v>
+        <v>90.954019999999986</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2728,14 +2728,14 @@
       <c r="H13" s="4"/>
     </row>
     <row r="15" spans="1:9" ht="14.25" customHeight="1">
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:9" s="5" customFormat="1" ht="28">
       <c r="A16" s="4" t="s">
@@ -3101,116 +3101,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743">
-      <UserInfo>
-        <DisplayName>Carlos Andres Lozano Garzon</DisplayName>
-        <AccountId>13</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Dario Ernesto Correal Torres</DisplayName>
-        <AccountId>15</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Mario  Fernando De la rosa Rosero</DisplayName>
-        <AccountId>16</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Christian Camilo Aparicio Baquen</DisplayName>
-        <AccountId>50</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Arturo Henao Chaparro</DisplayName>
-        <AccountId>48</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Luis Esteban Florez Salamanca</DisplayName>
-        <AccountId>33</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Ivan David Salazar Cardenas</DisplayName>
-        <AccountId>52</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Juan Carlos Marin Morales</DisplayName>
-        <AccountId>53</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Sofia Duque Gomez</DisplayName>
-        <AccountId>60</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Andres Felipe Romero Brand</DisplayName>
-        <AccountId>91</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lindsay Vanessa Pinto Morato</DisplayName>
-        <AccountId>92</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Miguel Angel Acosta Walteros</DisplayName>
-        <AccountId>94</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Juan David Diaz Ipuz</DisplayName>
-        <AccountId>90</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lily Aitana valentina Duque Chavez</DisplayName>
-        <AccountId>17</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Isaac David Bermudez Lara</DisplayName>
-        <AccountId>95</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Daniel Alejandro Angel Fuertes</DisplayName>
-        <AccountId>55</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jeniffer Liliam Mendoza Espinosa</DisplayName>
-        <AccountId>97</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Kevin Cohen Solano</DisplayName>
-        <AccountId>93</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cesar Luis Moreno Gonzalez</DisplayName>
-        <AccountId>96</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jose Cristobal Arroyo Castellanos</DisplayName>
-        <AccountId>54</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3463,21 +3359,122 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743">
+      <UserInfo>
+        <DisplayName>Carlos Andres Lozano Garzon</DisplayName>
+        <AccountId>13</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Dario Ernesto Correal Torres</DisplayName>
+        <AccountId>15</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Mario  Fernando De la rosa Rosero</DisplayName>
+        <AccountId>16</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Christian Camilo Aparicio Baquen</DisplayName>
+        <AccountId>50</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Arturo Henao Chaparro</DisplayName>
+        <AccountId>48</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Luis Esteban Florez Salamanca</DisplayName>
+        <AccountId>33</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Ivan David Salazar Cardenas</DisplayName>
+        <AccountId>52</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Juan Carlos Marin Morales</DisplayName>
+        <AccountId>53</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Sofia Duque Gomez</DisplayName>
+        <AccountId>60</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Andres Felipe Romero Brand</DisplayName>
+        <AccountId>91</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lindsay Vanessa Pinto Morato</DisplayName>
+        <AccountId>92</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Miguel Angel Acosta Walteros</DisplayName>
+        <AccountId>94</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Juan David Diaz Ipuz</DisplayName>
+        <AccountId>90</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lily Aitana valentina Duque Chavez</DisplayName>
+        <AccountId>17</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Isaac David Bermudez Lara</DisplayName>
+        <AccountId>95</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Daniel Alejandro Angel Fuertes</DisplayName>
+        <AccountId>55</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jeniffer Liliam Mendoza Espinosa</DisplayName>
+        <AccountId>97</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Kevin Cohen Solano</DisplayName>
+        <AccountId>93</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cesar Luis Moreno Gonzalez</DisplayName>
+        <AccountId>96</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jose Cristobal Arroyo Castellanos</DisplayName>
+        <AccountId>54</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
-    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3502,9 +3499,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
+    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
excel y word semicompletos
</commit_message>
<xml_diff>
--- a/Docs/ISIS1225-TablasDatosReto2.xlsx
+++ b/Docs/ISIS1225-TablasDatosReto2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f37e920cb68ed4a8/Desktop/Reto2-G03/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{4A5DBDDE-59DE-4983-A5DD-216DD4370536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3F9D279-734E-4354-9D33-39B9177A17B5}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{4A5DBDDE-59DE-4983-A5DD-216DD4370536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FED316B5-EBB6-4662-8D56-60A44B29479C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
@@ -1069,31 +1069,31 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>4.3148999214172319</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>6.1424201011657686</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>6.1981198310851999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>8.6322199821472143</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>10.21958003044127</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>11.634040021896318</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>13.982019996643022</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>13.683559942245441</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>17.169700002670218</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2395,7 +2395,7 @@
     <col min="1" max="1" width="19.1796875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="12" width="24.453125" customWidth="1"/>
   </cols>
@@ -2800,23 +2800,23 @@
         <v>20000</v>
       </c>
       <c r="C18" s="3">
-        <v>0</v>
+        <v>3.9840998649597101</v>
       </c>
       <c r="D18" s="3">
-        <v>0</v>
+        <v>4.8567998409271196</v>
       </c>
       <c r="E18" s="3">
-        <v>0</v>
+        <v>4.5381000041961599</v>
       </c>
       <c r="F18" s="3">
-        <v>0</v>
+        <v>4.1802999973297101</v>
       </c>
       <c r="G18" s="3">
-        <v>0</v>
+        <v>4.0151998996734601</v>
       </c>
       <c r="H18" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>4.3148999214172319</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2828,23 +2828,23 @@
         <v>30000</v>
       </c>
       <c r="C19" s="3">
-        <v>0</v>
+        <v>6.2367999553680402</v>
       </c>
       <c r="D19" s="3">
-        <v>0</v>
+        <v>6.29010009765625</v>
       </c>
       <c r="E19" s="3">
-        <v>0</v>
+        <v>6.2019002437591499</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>5.9577002525329501</v>
       </c>
       <c r="G19" s="3">
-        <v>0</v>
+        <v>6.0255999565124503</v>
       </c>
       <c r="H19" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>6.1424201011657686</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -2856,23 +2856,23 @@
         <v>40000</v>
       </c>
       <c r="C20" s="3">
-        <v>0</v>
+        <v>5.7714996337890598</v>
       </c>
       <c r="D20" s="3">
-        <v>0</v>
+        <v>6.2012999057769704</v>
       </c>
       <c r="E20" s="3">
-        <v>0</v>
+        <v>6.5951998233795104</v>
       </c>
       <c r="F20" s="3">
-        <v>0</v>
+        <v>6.1326999664306596</v>
       </c>
       <c r="G20" s="3">
-        <v>0</v>
+        <v>6.2898998260498002</v>
       </c>
       <c r="H20" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>6.1981198310851999</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -2884,23 +2884,23 @@
         <v>50000</v>
       </c>
       <c r="C21" s="3">
-        <v>0</v>
+        <v>7.7952001094818097</v>
       </c>
       <c r="D21" s="3">
-        <v>0</v>
+        <v>8.6152000427246094</v>
       </c>
       <c r="E21" s="3">
-        <v>0</v>
+        <v>9.1731998920440603</v>
       </c>
       <c r="F21" s="3">
-        <v>0</v>
+        <v>9.1158998012542707</v>
       </c>
       <c r="G21" s="3">
-        <v>0</v>
+        <v>8.4616000652313197</v>
       </c>
       <c r="H21" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>8.6322199821472143</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2912,23 +2912,23 @@
         <v>60000</v>
       </c>
       <c r="C22" s="3">
-        <v>0</v>
+        <v>8.6030998229980398</v>
       </c>
       <c r="D22" s="3">
-        <v>0</v>
+        <v>10.4917001724243</v>
       </c>
       <c r="E22" s="3">
-        <v>0</v>
+        <v>10.7696998119354</v>
       </c>
       <c r="F22" s="3">
-        <v>0</v>
+        <v>11.457000255584701</v>
       </c>
       <c r="G22" s="3">
-        <v>0</v>
+        <v>9.7764000892639107</v>
       </c>
       <c r="H22" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>10.21958003044127</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -2940,23 +2940,23 @@
         <v>70000</v>
       </c>
       <c r="C23" s="3">
-        <v>0</v>
+        <v>11.468099832534699</v>
       </c>
       <c r="D23" s="3">
-        <v>0</v>
+        <v>11.4037001132965</v>
       </c>
       <c r="E23" s="3">
-        <v>0</v>
+        <v>11.5676999092102</v>
       </c>
       <c r="F23" s="3">
-        <v>0</v>
+        <v>11.6924002170562</v>
       </c>
       <c r="G23" s="3">
-        <v>0</v>
+        <v>12.038300037383999</v>
       </c>
       <c r="H23" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>11.634040021896318</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2968,23 +2968,23 @@
         <v>80000</v>
       </c>
       <c r="C24" s="3">
-        <v>0</v>
+        <v>13.178200244903501</v>
       </c>
       <c r="D24" s="3">
-        <v>0</v>
+        <v>15.4297997951507</v>
       </c>
       <c r="E24" s="3">
-        <v>0</v>
+        <v>13.221599817275999</v>
       </c>
       <c r="F24" s="3">
-        <v>0</v>
+        <v>13.305999994277901</v>
       </c>
       <c r="G24" s="3">
-        <v>0</v>
+        <v>14.774500131607001</v>
       </c>
       <c r="H24" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>13.982019996643022</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2996,23 +2996,23 @@
         <v>90000</v>
       </c>
       <c r="C25" s="3">
-        <v>0</v>
+        <v>13.598699808120699</v>
       </c>
       <c r="D25" s="3">
-        <v>0</v>
+        <v>13.616600036621</v>
       </c>
       <c r="E25" s="3">
-        <v>0</v>
+        <v>13.5401000976562</v>
       </c>
       <c r="F25" s="3">
-        <v>0</v>
+        <v>13.613499879837001</v>
       </c>
       <c r="G25" s="3">
-        <v>0</v>
+        <v>14.048899888992301</v>
       </c>
       <c r="H25" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>13.683559942245441</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3024,23 +3024,23 @@
         <v>100000</v>
       </c>
       <c r="C26" s="3">
-        <v>0</v>
+        <v>15.988400220870901</v>
       </c>
       <c r="D26" s="3">
-        <v>0</v>
+        <v>18.136799812316799</v>
       </c>
       <c r="E26" s="3">
-        <v>0</v>
+        <v>16.9165999889373</v>
       </c>
       <c r="F26" s="3">
-        <v>0</v>
+        <v>16.169800043106001</v>
       </c>
       <c r="G26" s="3">
-        <v>0</v>
+        <v>18.636899948120099</v>
       </c>
       <c r="H26" s="4">
         <f>AVERAGE(Table13[[#This Row],[Tiempo 1]:[Tiempo 5]])</f>
-        <v>0</v>
+        <v>17.169700002670218</v>
       </c>
     </row>
   </sheetData>
@@ -3101,12 +3101,116 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743">
+      <UserInfo>
+        <DisplayName>Carlos Andres Lozano Garzon</DisplayName>
+        <AccountId>13</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Dario Ernesto Correal Torres</DisplayName>
+        <AccountId>15</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Mario  Fernando De la rosa Rosero</DisplayName>
+        <AccountId>16</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Christian Camilo Aparicio Baquen</DisplayName>
+        <AccountId>50</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Arturo Henao Chaparro</DisplayName>
+        <AccountId>48</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Luis Esteban Florez Salamanca</DisplayName>
+        <AccountId>33</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Ivan David Salazar Cardenas</DisplayName>
+        <AccountId>52</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Juan Carlos Marin Morales</DisplayName>
+        <AccountId>53</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Sofia Duque Gomez</DisplayName>
+        <AccountId>60</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Andres Felipe Romero Brand</DisplayName>
+        <AccountId>91</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lindsay Vanessa Pinto Morato</DisplayName>
+        <AccountId>92</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Miguel Angel Acosta Walteros</DisplayName>
+        <AccountId>94</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Juan David Diaz Ipuz</DisplayName>
+        <AccountId>90</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Lily Aitana valentina Duque Chavez</DisplayName>
+        <AccountId>17</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Isaac David Bermudez Lara</DisplayName>
+        <AccountId>95</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Daniel Alejandro Angel Fuertes</DisplayName>
+        <AccountId>55</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jeniffer Liliam Mendoza Espinosa</DisplayName>
+        <AccountId>97</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Kevin Cohen Solano</DisplayName>
+        <AccountId>93</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cesar Luis Moreno Gonzalez</DisplayName>
+        <AccountId>96</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jose Cristobal Arroyo Castellanos</DisplayName>
+        <AccountId>54</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3359,122 +3463,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743">
-      <UserInfo>
-        <DisplayName>Carlos Andres Lozano Garzon</DisplayName>
-        <AccountId>13</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Dario Ernesto Correal Torres</DisplayName>
-        <AccountId>15</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Mario  Fernando De la rosa Rosero</DisplayName>
-        <AccountId>16</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Christian Camilo Aparicio Baquen</DisplayName>
-        <AccountId>50</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Arturo Henao Chaparro</DisplayName>
-        <AccountId>48</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Luis Esteban Florez Salamanca</DisplayName>
-        <AccountId>33</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Ivan David Salazar Cardenas</DisplayName>
-        <AccountId>52</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Juan Carlos Marin Morales</DisplayName>
-        <AccountId>53</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Sofia Duque Gomez</DisplayName>
-        <AccountId>60</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Andres Felipe Romero Brand</DisplayName>
-        <AccountId>91</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lindsay Vanessa Pinto Morato</DisplayName>
-        <AccountId>92</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Miguel Angel Acosta Walteros</DisplayName>
-        <AccountId>94</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Juan David Diaz Ipuz</DisplayName>
-        <AccountId>90</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Lily Aitana valentina Duque Chavez</DisplayName>
-        <AccountId>17</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Isaac David Bermudez Lara</DisplayName>
-        <AccountId>95</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Daniel Alejandro Angel Fuertes</DisplayName>
-        <AccountId>55</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jeniffer Liliam Mendoza Espinosa</DisplayName>
-        <AccountId>97</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Kevin Cohen Solano</DisplayName>
-        <AccountId>93</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cesar Luis Moreno Gonzalez</DisplayName>
-        <AccountId>96</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jose Cristobal Arroyo Castellanos</DisplayName>
-        <AccountId>54</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
+    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3499,12 +3502,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
-    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>